<commit_message>
Update Beats data to April 2026
</commit_message>
<xml_diff>
--- a/data/Beats data .xlsx
+++ b/data/Beats data .xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8b6b0526c34ee03f/Documents/GEX/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8b6b0526c34ee03f/Documents/GEX/APP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1442F96C-265E-483F-8F9C-5E1D2509DB69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E6F969C6-3194-47CB-AC42-26B183CC9832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2955" yWindow="1185" windowWidth="24930" windowHeight="18405" xr2:uid="{BA5A99B9-B584-445B-86B3-7E1FE6C723EE}"/>
+    <workbookView xWindow="8970" yWindow="870" windowWidth="24930" windowHeight="18405" xr2:uid="{02F02110-25CA-4221-B112-74F432C584E1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -60,34 +60,34 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
+      <sz val="11"/>
+      <color rgb="FF242424"/>
+      <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FF242424"/>
-      <name val="Aptos"/>
+      <name val="Segoe UI"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -96,11 +96,13 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
-      <top style="medium">
+      <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom/>
@@ -108,6 +110,19 @@
     </border>
     <border>
       <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
@@ -118,14 +133,45 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
         <color rgb="FF000000"/>
       </right>
       <top/>
       <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
@@ -134,26 +180,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="17" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="17" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="17" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="10" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -487,347 +539,355 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A051D7C-E9F3-42DC-92C2-0C1D74F70F52}">
-  <dimension ref="B2:C46"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC291C8F-8D05-4823-ACFA-B515AEDD3ECD}">
+  <dimension ref="B3:C46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="13.5703125" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
-    </row>
-    <row r="4" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="2"/>
-    </row>
-    <row r="5" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="3"/>
+      <c r="C4" s="4"/>
+    </row>
+    <row r="5" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="4">
+    <row r="6" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="6">
         <v>44927</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="7">
         <v>1.01E-2</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="4">
+    <row r="7" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="6">
         <v>44958</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="7">
         <v>1.0800000000000001E-2</v>
       </c>
     </row>
-    <row r="8" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="4">
+    <row r="8" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="6">
         <v>44986</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="7">
         <v>2.23E-2</v>
       </c>
     </row>
-    <row r="9" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="4">
+    <row r="9" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="6">
         <v>45017</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="7">
         <v>1.5699999999999999E-2</v>
       </c>
     </row>
-    <row r="10" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="4">
+    <row r="10" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="6">
         <v>45047</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="7">
         <v>4.3099999999999999E-2</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="4">
+    <row r="11" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="6">
         <v>45078</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="7">
         <v>1.6400000000000001E-2</v>
       </c>
     </row>
-    <row r="12" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="4">
+    <row r="12" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="6">
         <v>45108</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="7">
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="13" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="4">
+    <row r="13" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="6">
         <v>45139</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="7">
         <v>2.0400000000000001E-2</v>
       </c>
     </row>
-    <row r="14" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="4">
+    <row r="14" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="6">
         <v>45170</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="7">
         <v>1.66E-2</v>
       </c>
     </row>
-    <row r="15" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="4">
+    <row r="15" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="6">
         <v>45200</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="7">
         <v>1.12E-2</v>
       </c>
     </row>
-    <row r="16" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="4">
+    <row r="16" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="6">
         <v>45231</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C16" s="7">
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="4">
+    <row r="17" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="6">
         <v>45261</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="7">
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="18" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="4">
+    <row r="18" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="6">
         <v>45292</v>
       </c>
-      <c r="C18" s="5">
+      <c r="C18" s="7">
         <v>2.0199999999999999E-2</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="4">
+    <row r="19" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="6">
         <v>45323</v>
       </c>
-      <c r="C19" s="5">
+      <c r="C19" s="7">
         <v>2.98E-2</v>
       </c>
     </row>
-    <row r="20" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="4">
+    <row r="20" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="6">
         <v>45352</v>
       </c>
-      <c r="C20" s="5">
+      <c r="C20" s="7">
         <v>1.12E-2</v>
       </c>
     </row>
-    <row r="21" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="4">
+    <row r="21" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="6">
         <v>45383</v>
       </c>
-      <c r="C21" s="5">
+      <c r="C21" s="7">
         <v>1.47E-2</v>
       </c>
     </row>
-    <row r="22" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="4">
+    <row r="22" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="6">
         <v>45413</v>
       </c>
-      <c r="C22" s="5">
+      <c r="C22" s="7">
         <v>8.9800000000000005E-2</v>
       </c>
     </row>
-    <row r="23" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="4">
+    <row r="23" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="6">
         <v>45444</v>
       </c>
-      <c r="C23" s="5">
+      <c r="C23" s="7">
         <v>2.1399999999999999E-2</v>
       </c>
     </row>
-    <row r="24" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="4">
+    <row r="24" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="6">
         <v>45474</v>
       </c>
-      <c r="C24" s="5">
+      <c r="C24" s="7">
         <v>2.6200000000000001E-2</v>
       </c>
     </row>
-    <row r="25" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="4">
+    <row r="25" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="6">
         <v>45505</v>
       </c>
-      <c r="C25" s="5">
+      <c r="C25" s="7">
         <v>5.5E-2</v>
       </c>
     </row>
-    <row r="26" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="4">
+    <row r="26" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="6">
         <v>45536</v>
       </c>
-      <c r="C26" s="5">
+      <c r="C26" s="7">
         <v>1.5299999999999999E-2</v>
       </c>
     </row>
-    <row r="27" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="4">
+    <row r="27" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="6">
         <v>45566</v>
       </c>
-      <c r="C27" s="5">
+      <c r="C27" s="7">
         <v>1.9400000000000001E-2</v>
       </c>
     </row>
-    <row r="28" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="4">
+    <row r="28" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="6">
         <v>45597</v>
       </c>
-      <c r="C28" s="5">
+      <c r="C28" s="7">
         <v>7.4099999999999999E-2</v>
       </c>
     </row>
-    <row r="29" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="4">
+    <row r="29" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="6">
         <v>45627</v>
       </c>
-      <c r="C29" s="5">
+      <c r="C29" s="7">
         <v>3.6900000000000002E-2</v>
       </c>
     </row>
-    <row r="30" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="4">
+    <row r="30" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="6">
         <v>45658</v>
       </c>
-      <c r="C30" s="5">
+      <c r="C30" s="7">
         <v>2.0799999999999999E-2</v>
       </c>
     </row>
-    <row r="31" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="4">
+    <row r="31" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="6">
         <v>45689</v>
       </c>
-      <c r="C31" s="5">
+      <c r="C31" s="7">
         <v>1.77E-2</v>
       </c>
     </row>
-    <row r="32" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="4">
+    <row r="32" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="6">
         <v>45717</v>
       </c>
-      <c r="C32" s="5">
+      <c r="C32" s="7">
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="33" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="4">
+    <row r="33" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="6">
         <v>45748</v>
       </c>
-      <c r="C33" s="5">
+      <c r="C33" s="7">
         <v>2.07E-2</v>
       </c>
     </row>
-    <row r="34" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="4">
+    <row r="34" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="6">
         <v>45778</v>
       </c>
-      <c r="C34" s="5">
+      <c r="C34" s="7">
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="35" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="4">
+    <row r="35" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="6">
         <v>45809</v>
       </c>
-      <c r="C35" s="5">
+      <c r="C35" s="7">
         <v>7.7399999999999997E-2</v>
       </c>
     </row>
-    <row r="36" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="4">
+    <row r="36" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="6">
         <v>45839</v>
       </c>
-      <c r="C36" s="5">
+      <c r="C36" s="7">
         <v>1.5699999999999999E-2</v>
       </c>
     </row>
-    <row r="37" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="4">
+    <row r="37" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="6">
         <v>45870</v>
       </c>
-      <c r="C37" s="5">
+      <c r="C37" s="7">
         <v>1.8100000000000002E-2</v>
       </c>
     </row>
-    <row r="38" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="4">
+    <row r="38" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="6">
         <v>45901</v>
       </c>
-      <c r="C38" s="5">
+      <c r="C38" s="7">
         <v>1.46E-2</v>
       </c>
     </row>
-    <row r="39" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="4">
+    <row r="39" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="6">
         <v>45931</v>
       </c>
-      <c r="C39" s="5">
+      <c r="C39" s="7">
         <v>1.7600000000000001E-2</v>
       </c>
     </row>
-    <row r="40" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="4">
+    <row r="40" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="6">
         <v>45962</v>
       </c>
-      <c r="C40" s="5">
+      <c r="C40" s="7">
         <v>2.3300000000000001E-2</v>
       </c>
     </row>
-    <row r="41" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="4">
+    <row r="41" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="6">
         <v>45992</v>
       </c>
-      <c r="C41" s="5">
+      <c r="C41" s="7">
         <v>1.83E-2</v>
       </c>
     </row>
-    <row r="42" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="4">
+    <row r="42" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B42" s="6">
         <v>46023</v>
       </c>
-      <c r="C42" s="5">
+      <c r="C42" s="7">
         <v>1.54E-2</v>
       </c>
     </row>
-    <row r="43" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="4">
+    <row r="43" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B43" s="6">
         <v>46054</v>
       </c>
-      <c r="C43" s="5">
+      <c r="C43" s="7">
         <v>1.44E-2</v>
       </c>
     </row>
-    <row r="44" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="4">
+    <row r="44" spans="2:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B44" s="6">
         <v>46082</v>
       </c>
-      <c r="C44" s="5">
+      <c r="C44" s="7">
         <v>6.4999999999999997E-3</v>
       </c>
     </row>
-    <row r="45" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="4">
+    <row r="45" spans="2:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B45" s="8">
         <v>46113</v>
       </c>
-      <c r="C45" s="5">
+      <c r="C45" s="9">
         <v>6.8999999999999999E-3</v>
       </c>
     </row>
-    <row r="46" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B46" s="6"/>
+    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C46" s="10">
+        <f>SUM(C18:C45)</f>
+        <v>0.74939999999999984</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>